<commit_message>
Papers to find: ISBNs of the books; NBS TN 993 found (free at NIST)
</commit_message>
<xml_diff>
--- a/docs/papers_to_find.xlsx
+++ b/docs/papers_to_find.xlsx
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -78,6 +78,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2781,12 +2782,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
@@ -2802,17 +2803,22 @@
           <t>کتاب / دیتاشیت</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>ISBN / لینک</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>داده‌ها</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>وضعیت</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>یادداشت</t>
         </is>
@@ -2829,11 +2835,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>نسخه‌ی انگلیسی: Handbook of Physical Quantities, CRC 1997, ISBN 0849328616 (978-0849328619)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>LiNbO3: انبساط گرمایی؛ LiTaO3: انبساط گرمایی؛ BaTiO3: انبساط گرمایی؛ GaAs: انبساط گرمایی؛ CdSe: انبساط گرمایی</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2846,11 +2855,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>LiB3O5: رسانش گرمایی؛ LiIO3: انبساط گرمایی</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2863,11 +2875,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>ISBN ندارد (پیش از ۱۹۸۷، کتاب شوروی)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>LiNbO3: رسانش گرمایی؛ KH2PO4: انبساط گرمایی؛ NH4H2PO4: انبساط گرمایی؛ Ag3AsS3: انبساط گرمایی</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -2878,17 +2893,17 @@
           <t>S.S. Ballard, J.S. Browder: Thermal Properties. In: CRC Handbook of Laser Science and Technology, Vol. IV, Optical Materials: Part 2, ed. by M.J. Weber (CRC Press, Boca Raton, 1987), pp. 49–54</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>LiNbO3: انبساط گرمایی؛ BaTiO3: رسانش گرمایی</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>در مجموعه هست</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Weber 1986، جلد IV بخش ۲، در مجموعه است؛ خودم می‌خوانم</t>
         </is>
@@ -2905,11 +2920,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>KTiOPO4: انبساط گرمایی؛ Li2B4O7: انبساط گرمایی</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2922,11 +2940,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>ISBN ندارد (پیش از ۱۹۸۷، کتاب شوروی)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>GaSe: انبساط گرمایی؛ Ag3AsS3: رسانش گرمایی؛ CdGeAs2: رسانش گرمایی</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2939,11 +2960,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>ISBN ندارد (پیش از ۱۹۸۷، کتاب شوروی)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>KH2PO4: رسانش گرمایی؛ NH4H2PO4: رسانش گرمایی؛ BaTiO3: رسانش گرمایی</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2956,11 +2980,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>ISBN 0582226295 (ویرایش ۱۶، Longman 1995)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>GaAs: انبساط گرمایی</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2971,38 +2998,51 @@
           <t>M. J. Dodge, in Handbook ofLaserScience andTechnology, Vol. IV, Optical Material; Part2, Refractive Index, M. J. Weber, Ed. (CRC Press, BocaRaton, 1986).</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>CaMoO4: dn/dT (منبع Bond)؛ PbMoO4: dn/dT (منبع Malitson)</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>در مجموعه هست</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Weber 1986، جلد IV بخش ۲، در مجموعه است؛ خودم می‌خوانم</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>A. Feldman, D. Horowitz, R. M. Waxler, andM. J. Dodge, Nat. Bur. Stand. (U.S.), Tech. Note 993, (Feb.. 1979).</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/Legacy/TN/nbstechnicalnote993.pdf (رایگان)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Al2O3: dn/dT (منبع Querry)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>پیدا شد</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>خودم دانلود کردم؛ لازم نیست بگردی</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>